<commit_message>
-created minimal example skeleton
</commit_message>
<xml_diff>
--- a/tutorials/data/input_chp.xlsx
+++ b/tutorials/data/input_chp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1_PROJEKTI\2_SENERGYNETS_in_corso\4_Code\8_pandaprosumer_rep5\tutorials\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eprade\Git\pandaprosumer_OS\tutorials\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64560B5D-A734-4737-8308-1C3CA0F54376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E971F5D7-EAD8-4E09-940D-C66394558543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -78,7 +78,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -96,7 +96,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="de-DE"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -447,9 +447,6 @@
                 <c:pt idx="95">
                   <c:v>0.98958333333333304</c:v>
                 </c:pt>
-                <c:pt idx="96">
-                  <c:v>1</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -745,9 +742,6 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="96">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -913,6 +907,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -920,7 +915,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1803,7 +1797,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D290"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.5703125" customWidth="1"/>
@@ -1830,7 +1824,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="2">
         <v>273</v>
@@ -1844,7 +1838,7 @@
         <v>1.0416666666666666E-2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="2">
         <v>273</v>
@@ -1858,7 +1852,7 @@
         <v>2.0833333333333301E-2</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" s="2">
         <v>273</v>
@@ -1872,7 +1866,7 @@
         <v>3.125E-2</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" s="2">
         <v>273</v>
@@ -1886,7 +1880,7 @@
         <v>4.1666666666666699E-2</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" s="2">
         <v>273</v>
@@ -1900,7 +1894,7 @@
         <v>5.2083333333333301E-2</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="2">
         <v>273</v>
@@ -1914,7 +1908,7 @@
         <v>6.25E-2</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8" s="2">
         <v>273</v>
@@ -1928,7 +1922,7 @@
         <v>7.2916666666666699E-2</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="2">
         <v>273</v>
@@ -1942,7 +1936,7 @@
         <v>8.3333333333333301E-2</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" s="2">
         <v>273</v>
@@ -1956,7 +1950,7 @@
         <v>9.375E-2</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" s="2">
         <v>273</v>
@@ -1970,7 +1964,7 @@
         <v>0.104166666666667</v>
       </c>
       <c r="B12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" s="2">
         <v>273</v>
@@ -1984,7 +1978,7 @@
         <v>0.114583333333333</v>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C13" s="2">
         <v>273</v>
@@ -1998,7 +1992,7 @@
         <v>0.125</v>
       </c>
       <c r="B14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C14" s="2">
         <v>273</v>
@@ -2012,7 +2006,7 @@
         <v>0.13541666666666699</v>
       </c>
       <c r="B15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C15" s="2">
         <v>273</v>
@@ -2026,7 +2020,7 @@
         <v>0.14583333333333301</v>
       </c>
       <c r="B16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" s="2">
         <v>273</v>
@@ -2040,7 +2034,7 @@
         <v>0.15625</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" s="2">
         <v>273</v>
@@ -2054,7 +2048,7 @@
         <v>0.16666666666666699</v>
       </c>
       <c r="B18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" s="2">
         <v>273</v>
@@ -2068,7 +2062,7 @@
         <v>0.17708333333333301</v>
       </c>
       <c r="B19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" s="2">
         <v>273</v>
@@ -2082,7 +2076,7 @@
         <v>0.1875</v>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" s="2">
         <v>273</v>
@@ -2096,7 +2090,7 @@
         <v>0.19791666666666699</v>
       </c>
       <c r="B21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" s="2">
         <v>273</v>
@@ -2110,7 +2104,7 @@
         <v>0.20833333333333301</v>
       </c>
       <c r="B22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" s="2">
         <v>273</v>
@@ -2124,7 +2118,7 @@
         <v>0.21875</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C23" s="2">
         <v>273</v>
@@ -2138,7 +2132,7 @@
         <v>0.22916666666666699</v>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24" s="2">
         <v>273</v>
@@ -2152,7 +2146,7 @@
         <v>0.23958333333333301</v>
       </c>
       <c r="B25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" s="2">
         <v>273</v>
@@ -2166,7 +2160,7 @@
         <v>0.25</v>
       </c>
       <c r="B26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C26" s="2">
         <v>273</v>
@@ -2180,7 +2174,7 @@
         <v>0.26041666666666702</v>
       </c>
       <c r="B27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" s="2">
         <v>273</v>
@@ -2194,7 +2188,7 @@
         <v>0.27083333333333298</v>
       </c>
       <c r="B28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C28" s="2">
         <v>273</v>
@@ -2208,7 +2202,7 @@
         <v>0.28125</v>
       </c>
       <c r="B29">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C29" s="2">
         <v>273</v>
@@ -2222,7 +2216,7 @@
         <v>0.29166666666666702</v>
       </c>
       <c r="B30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C30" s="2">
         <v>273</v>
@@ -2236,7 +2230,7 @@
         <v>0.30208333333333298</v>
       </c>
       <c r="B31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C31" s="2">
         <v>278</v>
@@ -2250,7 +2244,7 @@
         <v>0.3125</v>
       </c>
       <c r="B32">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C32" s="2">
         <v>278</v>
@@ -2264,7 +2258,7 @@
         <v>0.32291666666666702</v>
       </c>
       <c r="B33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C33" s="2">
         <v>278</v>
@@ -2278,7 +2272,7 @@
         <v>0.33333333333333298</v>
       </c>
       <c r="B34">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C34" s="2">
         <v>278</v>
@@ -2292,7 +2286,7 @@
         <v>0.34375</v>
       </c>
       <c r="B35">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C35" s="2">
         <v>278</v>
@@ -2306,7 +2300,7 @@
         <v>0.35416666666666702</v>
       </c>
       <c r="B36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36" s="2">
         <v>278</v>
@@ -2320,7 +2314,7 @@
         <v>0.36458333333333298</v>
       </c>
       <c r="B37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C37" s="2">
         <v>278</v>
@@ -2334,7 +2328,7 @@
         <v>0.375</v>
       </c>
       <c r="B38">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C38" s="2">
         <v>278</v>
@@ -2348,7 +2342,7 @@
         <v>0.38541666666666702</v>
       </c>
       <c r="B39">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C39" s="2">
         <v>278</v>
@@ -2362,7 +2356,7 @@
         <v>0.39583333333333298</v>
       </c>
       <c r="B40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" s="2">
         <v>278</v>
@@ -2376,7 +2370,7 @@
         <v>0.40625</v>
       </c>
       <c r="B41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C41" s="2">
         <v>300</v>
@@ -2390,7 +2384,7 @@
         <v>0.41666666666666702</v>
       </c>
       <c r="B42">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C42" s="2">
         <v>300</v>
@@ -2404,7 +2398,7 @@
         <v>0.42708333333333298</v>
       </c>
       <c r="B43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C43" s="2">
         <v>300</v>
@@ -2418,7 +2412,7 @@
         <v>0.4375</v>
       </c>
       <c r="B44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C44" s="2">
         <v>300</v>
@@ -2432,7 +2426,7 @@
         <v>0.44791666666666702</v>
       </c>
       <c r="B45">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C45" s="2">
         <v>300</v>
@@ -2446,7 +2440,7 @@
         <v>0.45833333333333298</v>
       </c>
       <c r="B46">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C46" s="2">
         <v>300</v>
@@ -2460,7 +2454,7 @@
         <v>0.46875</v>
       </c>
       <c r="B47">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C47" s="2">
         <v>300</v>
@@ -2474,7 +2468,7 @@
         <v>0.47916666666666702</v>
       </c>
       <c r="B48">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C48" s="2">
         <v>300</v>
@@ -2488,7 +2482,7 @@
         <v>0.48958333333333298</v>
       </c>
       <c r="B49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C49" s="2">
         <v>300</v>
@@ -2502,7 +2496,7 @@
         <v>0.5</v>
       </c>
       <c r="B50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" s="2">
         <v>300</v>
@@ -2516,7 +2510,7 @@
         <v>0.51041666666666696</v>
       </c>
       <c r="B51">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C51" s="2">
         <v>300</v>
@@ -2530,7 +2524,7 @@
         <v>0.52083333333333304</v>
       </c>
       <c r="B52">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C52" s="2">
         <v>300</v>
@@ -2544,7 +2538,7 @@
         <v>0.53125</v>
       </c>
       <c r="B53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C53" s="2">
         <v>300</v>
@@ -2558,7 +2552,7 @@
         <v>0.54166666666666696</v>
       </c>
       <c r="B54">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" s="2">
         <v>300</v>
@@ -2572,7 +2566,7 @@
         <v>0.55208333333333304</v>
       </c>
       <c r="B55">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" s="2">
         <v>300</v>
@@ -2586,7 +2580,7 @@
         <v>0.5625</v>
       </c>
       <c r="B56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C56" s="2">
         <v>300</v>
@@ -2600,7 +2594,7 @@
         <v>0.57291666666666696</v>
       </c>
       <c r="B57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C57" s="2">
         <v>300</v>
@@ -2614,7 +2608,7 @@
         <v>0.58333333333333304</v>
       </c>
       <c r="B58">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C58" s="2">
         <v>300</v>
@@ -2628,7 +2622,7 @@
         <v>0.59375</v>
       </c>
       <c r="B59">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C59" s="2">
         <v>300</v>
@@ -2642,7 +2636,7 @@
         <v>0.60416666666666696</v>
       </c>
       <c r="B60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C60" s="2">
         <v>300</v>
@@ -2656,7 +2650,7 @@
         <v>0.61458333333333304</v>
       </c>
       <c r="B61">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C61" s="2">
         <v>300</v>
@@ -2670,7 +2664,7 @@
         <v>0.625</v>
       </c>
       <c r="B62">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C62" s="2">
         <v>300</v>
@@ -2684,7 +2678,7 @@
         <v>0.63541666666666696</v>
       </c>
       <c r="B63">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C63" s="2">
         <v>300</v>
@@ -2698,7 +2692,7 @@
         <v>0.64583333333333304</v>
       </c>
       <c r="B64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C64" s="2">
         <v>300</v>
@@ -2712,7 +2706,7 @@
         <v>0.65625</v>
       </c>
       <c r="B65">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C65" s="2">
         <v>300</v>
@@ -2726,7 +2720,7 @@
         <v>0.66666666666666696</v>
       </c>
       <c r="B66">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C66" s="2">
         <v>300</v>
@@ -2740,7 +2734,7 @@
         <v>0.67708333333333304</v>
       </c>
       <c r="B67">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C67" s="2">
         <v>300</v>
@@ -2754,7 +2748,7 @@
         <v>0.6875</v>
       </c>
       <c r="B68">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C68" s="2">
         <v>300</v>
@@ -2768,7 +2762,7 @@
         <v>0.69791666666666696</v>
       </c>
       <c r="B69">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C69" s="2">
         <v>300</v>
@@ -2782,7 +2776,7 @@
         <v>0.70833333333333304</v>
       </c>
       <c r="B70">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C70" s="2">
         <v>300</v>
@@ -2796,7 +2790,7 @@
         <v>0.71875</v>
       </c>
       <c r="B71">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C71" s="2">
         <v>300</v>
@@ -2810,7 +2804,7 @@
         <v>0.72916666666666696</v>
       </c>
       <c r="B72">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C72" s="2">
         <v>300</v>
@@ -2824,7 +2818,7 @@
         <v>0.73958333333333304</v>
       </c>
       <c r="B73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C73" s="2">
         <v>300</v>
@@ -2838,7 +2832,7 @@
         <v>0.75</v>
       </c>
       <c r="B74">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C74" s="2">
         <v>300</v>
@@ -2852,7 +2846,7 @@
         <v>0.76041666666666696</v>
       </c>
       <c r="B75">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C75" s="2">
         <v>273</v>
@@ -2866,7 +2860,7 @@
         <v>0.77083333333333304</v>
       </c>
       <c r="B76">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C76" s="2">
         <v>273</v>
@@ -2880,7 +2874,7 @@
         <v>0.78125</v>
       </c>
       <c r="B77">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C77" s="2">
         <v>273</v>
@@ -2894,7 +2888,7 @@
         <v>0.79166666666666696</v>
       </c>
       <c r="B78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C78" s="2">
         <v>273</v>
@@ -2908,7 +2902,7 @@
         <v>0.80208333333333304</v>
       </c>
       <c r="B79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C79" s="2">
         <v>273</v>
@@ -2922,7 +2916,7 @@
         <v>0.8125</v>
       </c>
       <c r="B80">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C80" s="2">
         <v>273</v>
@@ -2936,7 +2930,7 @@
         <v>0.82291666666666696</v>
       </c>
       <c r="B81">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C81" s="2">
         <v>273</v>
@@ -2950,7 +2944,7 @@
         <v>0.83333333333333304</v>
       </c>
       <c r="B82">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C82" s="2">
         <v>273</v>
@@ -2964,7 +2958,7 @@
         <v>0.84375</v>
       </c>
       <c r="B83">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C83" s="2">
         <v>273</v>
@@ -2978,7 +2972,7 @@
         <v>0.85416666666666696</v>
       </c>
       <c r="B84">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C84" s="2">
         <v>273</v>
@@ -2992,7 +2986,7 @@
         <v>0.86458333333333304</v>
       </c>
       <c r="B85">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C85" s="2">
         <v>273</v>
@@ -3006,7 +3000,7 @@
         <v>0.875</v>
       </c>
       <c r="B86">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C86" s="2">
         <v>273</v>
@@ -3020,7 +3014,7 @@
         <v>0.88541666666666696</v>
       </c>
       <c r="B87">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C87" s="2">
         <v>273</v>
@@ -3034,7 +3028,7 @@
         <v>0.89583333333333304</v>
       </c>
       <c r="B88">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C88" s="2">
         <v>273</v>
@@ -3048,7 +3042,7 @@
         <v>0.90625</v>
       </c>
       <c r="B89">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C89" s="2">
         <v>273</v>
@@ -3062,7 +3056,7 @@
         <v>0.91666666666666696</v>
       </c>
       <c r="B90">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C90" s="2">
         <v>273</v>
@@ -3076,7 +3070,7 @@
         <v>0.92708333333333304</v>
       </c>
       <c r="B91">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C91" s="2">
         <v>273</v>
@@ -3090,7 +3084,7 @@
         <v>0.9375</v>
       </c>
       <c r="B92">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C92" s="2">
         <v>273</v>
@@ -3104,7 +3098,7 @@
         <v>0.94791666666666696</v>
       </c>
       <c r="B93">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C93" s="2">
         <v>273</v>
@@ -3118,7 +3112,7 @@
         <v>0.95833333333333304</v>
       </c>
       <c r="B94">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C94" s="2">
         <v>273</v>
@@ -3132,7 +3126,7 @@
         <v>0.96875</v>
       </c>
       <c r="B95">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C95" s="2">
         <v>273</v>
@@ -3146,7 +3140,7 @@
         <v>0.97916666666666696</v>
       </c>
       <c r="B96">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C96" s="2">
         <v>273</v>
@@ -3160,7 +3154,7 @@
         <v>0.98958333333333304</v>
       </c>
       <c r="B97">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C97" s="2">
         <v>273</v>
@@ -3170,18 +3164,8 @@
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="1">
-        <v>1</v>
-      </c>
-      <c r="B98">
-        <v>2</v>
-      </c>
-      <c r="C98" s="2">
-        <v>273</v>
-      </c>
-      <c r="D98">
-        <v>0</v>
-      </c>
+      <c r="A98" s="1"/>
+      <c r="C98" s="2"/>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="1"/>

</xml_diff>